<commit_message>
Adding login & points
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>CHROME</t>
   </si>
@@ -44,15 +44,9 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Guarda coins</t>
-  </si>
-  <si>
     <t>Ghost game</t>
   </si>
   <si>
-    <t>Registro.php</t>
-  </si>
-  <si>
     <t>Login.php</t>
   </si>
   <si>
@@ -72,6 +66,15 @@
   </si>
   <si>
     <t>Nuevo dino</t>
+  </si>
+  <si>
+    <t>BBDD</t>
+  </si>
+  <si>
+    <t>Guardar Coins</t>
+  </si>
+  <si>
+    <t>Register.php</t>
   </si>
 </sst>
 </file>
@@ -167,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -186,6 +189,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,7 +542,7 @@
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -566,10 +570,10 @@
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -595,52 +599,57 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v1 -Login & Points
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>CHROME</t>
   </si>
@@ -71,10 +71,13 @@
     <t>BBDD</t>
   </si>
   <si>
-    <t>Guardar Coins</t>
-  </si>
-  <si>
     <t>Register.php</t>
+  </si>
+  <si>
+    <t>ON GOING</t>
+  </si>
+  <si>
+    <t>Guardar Punts</t>
   </si>
 </sst>
 </file>
@@ -120,7 +123,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -154,6 +157,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -170,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -190,12 +199,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCCFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -486,7 +509,6 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -518,7 +540,9 @@
       <c r="C2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="11" t="s">
+        <v>16</v>
+      </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -546,7 +570,7 @@
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
-      <c r="D3" s="3"/>
+      <c r="D3" s="6"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -599,27 +623,31 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>8</v>
       </c>
+      <c r="E5" s="13"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" s="12" t="s">
         <v>8</v>
       </c>
+      <c r="E6" s="13"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="D7" s="12" t="s">
         <v>8</v>
       </c>
+      <c r="E7" s="13"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -635,6 +663,7 @@
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">

</xml_diff>

<commit_message>
v1 - Login & Register
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI-GF75thin\Desktop\PRATICAS GITHUB(Sistemas 0483-Program 0485-Entorns 0487)\DINO CHROME 2.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\DINO_CHROME_2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t>CHROME</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Guardar Punts</t>
+  </si>
+  <si>
+    <t>✓</t>
   </si>
 </sst>
 </file>
@@ -179,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -208,6 +211,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -596,7 +603,7 @@
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="3"/>
@@ -625,18 +632,20 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>8</v>
-      </c>
+      <c r="C5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="14"/>
       <c r="E5" s="13"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>8</v>
-      </c>
+      <c r="C6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="14"/>
       <c r="E6" s="13"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>